<commit_message>
tests: update reference data
</commit_message>
<xml_diff>
--- a/tests/eindhoven-500/reference/resultaten/werk/alle groepen/herkomsten/restdag/Pot_totaalproduct_OV.xlsx
+++ b/tests/eindhoven-500/reference/resultaten/werk/alle groepen/herkomsten/restdag/Pot_totaalproduct_OV.xlsx
@@ -1779,7 +1779,7 @@
         <v>83</v>
       </c>
       <c r="B84">
-        <v>633028.6891431372</v>
+        <v>633028.6891431373</v>
       </c>
       <c r="C84">
         <v>692418.0891014148</v>
@@ -6865,7 +6865,7 @@
         <v>2512577.529320225</v>
       </c>
       <c r="C383">
-        <v>3536745.100842435</v>
+        <v>3536745.100842436</v>
       </c>
       <c r="D383">
         <v>4796131.381436289</v>

</xml_diff>